<commit_message>
Proteger datos personales: RLS por columna, TTL de ubicaciones y política (T6)
- 0006: contact y occupancy fuera del grant de SELECT de authenticated
  (grant por columna: ninguna política futura puede exponerlos por
  accidente); consentimiento obligatorio para status on_mission
  (constraint) y borrado automático de brigade_locations > 24 h con
  pg_cron. Aplicada en remoto y verificada.
- Formulario: aviso de privacidad completo + confirmación obligatoria de
  haberlo comunicado al ocupante (queda como evidencia en Kobo).
- docs/politica-datos.md: borrador de política de tratamiento con modelo
  Responsable/Encargado, transferencia internacional, derechos, retención
  y pendientes antes de operar con datos reales.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/kobo/ais.xlsx
+++ b/kobo/ais.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -548,7 +548,7 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Esta inspección registra ubicación, características y fotos de la edificación para priorizar la evaluación estructural post-sismo. Los datos se tratan bajo la Ley 1581 de 2012.</t>
+          <t>AVISO DE PRIVACIDAD — Esta inspección registra ubicación, características y fotografías de la edificación (solo exteriores y elementos estructurales, no personas ni interiores habitados salvo lo estrictamente necesario) para priorizar la evaluación estructural post-sismo. Tratamiento según la Ley 1581 de 2012; política completa disponible con la entidad coordinadora. La clasificación resultante es un insumo de priorización: la habilitación definitiva es competencia de las autoridades.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -557,12 +557,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>select_one tipos_inspeccion</t>
+          <t>select_one confirmaciones</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>tipo_inspeccion</t>
+          <t>aviso_comunicado</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -576,21 +576,25 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Tipo de inspección</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
+          <t>¿Informaste al ocupante o responsable del inmueble el propósito de la inspección y el aviso de privacidad?</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Si no hay nadie presente, marca «No aplica (inmueble desocupado o sin acceso)»</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>select_one motivos_no_inspeccion</t>
+          <t>select_one tipos_inspeccion</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>motivo_no_inspeccion</t>
+          <t>tipo_inspeccion</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -599,16 +603,12 @@
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>${tipo_inspeccion} = 'no_inspeccionada'</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>¿Por qué no se inspeccionó?</t>
+          <t>Tipo de inspección</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -617,12 +617,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>select_one comunas</t>
+          <t>select_one motivos_no_inspeccion</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>comuna</t>
+          <t>motivo_no_inspeccion</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -630,17 +630,17 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>minimal</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>${tipo_inspeccion} = 'no_inspeccionada'</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Comuna</t>
+          <t>¿Por qué no se inspeccionó?</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -649,29 +649,33 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one comunas</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>barrio</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
+          <t>comuna</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>minimal</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Barrio</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Nombre del barrio dentro de la comuna</t>
-        </is>
-      </c>
+          <t>Comuna</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
@@ -682,7 +686,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>id_catastral</t>
+          <t>barrio</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -692,12 +696,12 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Identificación catastral</t>
+          <t>Barrio</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>sector-manzana-predio-mejora (IGAC), si se conoce</t>
+          <t>Nombre del barrio dentro de la comuna</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -710,26 +714,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>direccion</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>id_catastral</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Dirección de la edificación</t>
+          <t>Identificación catastral</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Como aparece en la placa, o la más aproximada</t>
+          <t>sector-manzana-predio-mejora (IGAC), si se conoce</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -742,63 +742,63 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>nombre_edificacion</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
+          <t>direccion</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Nombre de la edificación (si tiene)</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr"/>
+          <t>Dirección de la edificación</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Como aparece en la placa, o la más aproximada</t>
+        </is>
+      </c>
       <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>geopoint</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>gps</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>nombre_edificacion</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Ubicación GPS</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Capturar de pie frente a la edificación, con cielo visible</t>
-        </is>
-      </c>
+          <t>Nombre de la edificación (si tiene)</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>geopoint</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>pisos_sobre</t>
+          <t>gps</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -807,28 +807,20 @@
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada'</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>. &gt;= 1 and . &lt;= 50</t>
-        </is>
-      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Niveles sobre el terreno</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Debe estar entre 1 y 50</t>
-        </is>
-      </c>
+          <t>Ubicación GPS</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Capturar de pie frente a la edificación, con cielo visible</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -838,10 +830,14 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>sotanos</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
+          <t>pisos_sobre</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
@@ -850,57 +846,57 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>. &gt;= 0 and . &lt;= 10</t>
+          <t>. &gt;= 1 and . &lt;= 50</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Sótanos</t>
+          <t>Niveles sobre el terreno</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Debe estar entre 0 y 10</t>
+          <t>Debe estar entre 1 y 50</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>select_one usos</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>uso_predominante</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>minimal</t>
-        </is>
-      </c>
+          <t>sotanos</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>${tipo_inspeccion} != 'no_inspeccionada'</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 10</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Uso predominante de la edificación</t>
+          <t>Sótanos</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Debe estar entre 0 y 10</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -910,10 +906,14 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>uso_planta_baja</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
+          <t>uso_predominante</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>minimal</t>
@@ -928,7 +928,7 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Uso de la planta baja</t>
+          <t>Uso predominante de la edificación</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
@@ -937,38 +937,34 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>select_one usos</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>frente_m</t>
+          <t>uso_planta_baja</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>minimal</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr">
         <is>
           <t>${tipo_inspeccion} != 'no_inspeccionada'</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>. &gt; 0 and . &lt; 1000</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Frente aproximado (m)</t>
+          <t>Uso de la planta baja</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>Valor en metros, mayor que 0</t>
-        </is>
-      </c>
+      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -978,7 +974,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>fondo_m</t>
+          <t>frente_m</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -996,7 +992,7 @@
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Fondo aproximado (m)</t>
+          <t>Frente aproximado (m)</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
@@ -1009,51 +1005,55 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>select_one sistemas_estructurales</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>sistema_estructural</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>minimal</t>
-        </is>
-      </c>
+          <t>fondo_m</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
           <t>${tipo_inspeccion} != 'no_inspeccionada'</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>. &gt; 0 and . &lt; 1000</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Sistema estructural</t>
+          <t>Fondo aproximado (m)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Valor en metros, mayor que 0</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>select_one tipos_entrepiso</t>
+          <t>select_one sistemas_estructurales</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>tipo_entrepiso</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
+          <t>sistema_estructural</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
           <t>minimal</t>
@@ -1068,7 +1068,7 @@
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Tipo de entrepiso</t>
+          <t>Sistema estructural</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
@@ -1077,20 +1077,20 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>select_one rangos_ano</t>
+          <t>select_one tipos_entrepiso</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>rango_ano</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr"/>
+          <t>tipo_entrepiso</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>minimal</t>
+        </is>
+      </c>
       <c r="E22" t="inlineStr">
         <is>
           <t>${tipo_inspeccion} != 'no_inspeccionada'</t>
@@ -1100,7 +1100,7 @@
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Año de construcción</t>
+          <t>Tipo de entrepiso</t>
         </is>
       </c>
       <c r="I22" t="inlineStr"/>
@@ -1109,12 +1109,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>select_one colapsos</t>
+          <t>select_one rangos_ano</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>colapso</t>
+          <t>rango_ano</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1132,7 +1132,7 @@
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Colapso</t>
+          <t>Año de construcción</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -1141,12 +1141,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>select_one inclinaciones</t>
+          <t>select_one colapsos</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>inclinacion</t>
+          <t>colapso</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1164,7 +1164,7 @@
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Inclinación de la edificación o de un piso</t>
+          <t>Colapso</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
@@ -1173,12 +1173,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one inclinaciones</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>piso_mayor_dano</t>
+          <t>inclinacion</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1189,40 +1189,28 @@
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and ${colapso} != 'total'</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>. &gt;= 0 and . &lt;= 50</t>
-        </is>
-      </c>
+          <t>${tipo_inspeccion} != 'no_inspeccionada'</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
-          <t>¿Cuál es el piso de mayor daño?</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>La matriz de daño se evalúa en ese piso</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>0 = sótano; máximo 50</t>
-        </is>
-      </c>
+          <t>Inclinación de la edificación o de un piso</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>select_one niveles_dano</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>dano_vigas</t>
+          <t>piso_mayor_dano</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1233,28 +1221,40 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42')</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr"/>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and ${colapso} != 'total'</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 50</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Daño en vigas</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
+          <t>¿Cuál es el piso de mayor daño?</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>La matriz de daño se evalúa en ese piso</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>0 = sótano; máximo 50</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one niveles_dano</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>dano_vigas_pct</t>
+          <t>dano_vigas</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1265,36 +1265,28 @@
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42') and ${dano_vigas} != 'ninguno'</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>. &gt;= 1 and . &lt;= 100</t>
-        </is>
-      </c>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42')</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
-          <t>% de extensión del daño en vigas</t>
+          <t>Daño en vigas</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>Debe estar entre 1 y 100</t>
-        </is>
-      </c>
+      <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>select_one niveles_dano</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>dano_columnas</t>
+          <t>dano_vigas_pct</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1305,28 +1297,36 @@
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42')</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr"/>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42') and ${dano_vigas} != 'ninguno'</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>. &gt;= 1 and . &lt;= 100</t>
+        </is>
+      </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Daño en columnas</t>
+          <t>% de extensión del daño en vigas</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Debe estar entre 1 y 100</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one niveles_dano</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>dano_columnas_pct</t>
+          <t>dano_columnas</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1337,36 +1337,28 @@
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42') and ${dano_columnas} != 'ninguno'</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>. &gt;= 1 and . &lt;= 100</t>
-        </is>
-      </c>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42')</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
-          <t>% de extensión del daño en columnas</t>
+          <t>Daño en columnas</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>Debe estar entre 1 y 100</t>
-        </is>
-      </c>
+      <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>select_one niveles_dano</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>dano_nudos</t>
+          <t>dano_columnas_pct</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1377,28 +1369,36 @@
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14')</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr"/>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42') and ${dano_columnas} != 'ninguno'</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>. &gt;= 1 and . &lt;= 100</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Daño en nudos (unión viga-columna)</t>
+          <t>% de extensión del daño en columnas</t>
         </is>
       </c>
       <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Debe estar entre 1 y 100</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one niveles_dano</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>dano_nudos_pct</t>
+          <t>dano_nudos</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1409,36 +1409,28 @@
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14') and ${dano_nudos} != 'ninguno'</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>. &gt;= 1 and . &lt;= 100</t>
-        </is>
-      </c>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14')</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
-          <t>% de extensión del daño en nudos (unión viga-columna)</t>
+          <t>Daño en nudos (unión viga-columna)</t>
         </is>
       </c>
       <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>Debe estar entre 1 y 100</t>
-        </is>
-      </c>
+      <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>select_one niveles_dano</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>dano_conexiones</t>
+          <t>dano_nudos_pct</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1449,28 +1441,36 @@
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42')</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr"/>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14') and ${dano_nudos} != 'ninguno'</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>. &gt;= 1 and . &lt;= 100</t>
+        </is>
+      </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Daño en conexiones</t>
+          <t>% de extensión del daño en nudos (unión viga-columna)</t>
         </is>
       </c>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Debe estar entre 1 y 100</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one niveles_dano</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>dano_conexiones_pct</t>
+          <t>dano_conexiones</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1481,36 +1481,28 @@
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42') and ${dano_conexiones} != 'ninguno'</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>. &gt;= 1 and . &lt;= 100</t>
-        </is>
-      </c>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42')</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
-          <t>% de extensión del daño en conexiones</t>
+          <t>Daño en conexiones</t>
         </is>
       </c>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>Debe estar entre 1 y 100</t>
-        </is>
-      </c>
+      <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>select_one niveles_dano</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>dano_muros</t>
+          <t>dano_conexiones_pct</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1521,28 +1513,36 @@
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '12' or ${sistema_estructural} = '13')</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr"/>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42') and ${dano_conexiones} != 'ninguno'</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>. &gt;= 1 and . &lt;= 100</t>
+        </is>
+      </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Daño en muros estructurales</t>
+          <t>% de extensión del daño en conexiones</t>
         </is>
       </c>
       <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Debe estar entre 1 y 100</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one niveles_dano</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>dano_muros_pct</t>
+          <t>dano_muros</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1553,36 +1553,28 @@
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '12' or ${sistema_estructural} = '13') and ${dano_muros} != 'ninguno'</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>. &gt;= 1 and . &lt;= 100</t>
-        </is>
-      </c>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '12' or ${sistema_estructural} = '13')</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
-          <t>% de extensión del daño en muros estructurales</t>
+          <t>Daño en muros estructurales</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>Debe estar entre 1 y 100</t>
-        </is>
-      </c>
+      <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>select_one niveles_dano</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>dano_muros_portantes</t>
+          <t>dano_muros_pct</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1593,28 +1585,36 @@
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21' or ${sistema_estructural} = '22' or ${sistema_estructural} = '23' or ${sistema_estructural} = '51' or ${sistema_estructural} = '52' or ${sistema_estructural} = '50' or ${sistema_estructural} = '60')</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr"/>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '12' or ${sistema_estructural} = '13') and ${dano_muros} != 'ninguno'</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>. &gt;= 1 and . &lt;= 100</t>
+        </is>
+      </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Daño en muros portantes</t>
+          <t>% de extensión del daño en muros estructurales</t>
         </is>
       </c>
       <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Debe estar entre 1 y 100</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one niveles_dano</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>dano_muros_portantes_pct</t>
+          <t>dano_muros_portantes</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1625,36 +1625,28 @@
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21' or ${sistema_estructural} = '22' or ${sistema_estructural} = '23' or ${sistema_estructural} = '51' or ${sistema_estructural} = '52' or ${sistema_estructural} = '50' or ${sistema_estructural} = '60') and ${dano_muros_portantes} != 'ninguno'</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>. &gt;= 1 and . &lt;= 100</t>
-        </is>
-      </c>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21' or ${sistema_estructural} = '22' or ${sistema_estructural} = '23' or ${sistema_estructural} = '51' or ${sistema_estructural} = '52' or ${sistema_estructural} = '50' or ${sistema_estructural} = '60')</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
-          <t>% de extensión del daño en muros portantes</t>
+          <t>Daño en muros portantes</t>
         </is>
       </c>
       <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>Debe estar entre 1 y 100</t>
-        </is>
-      </c>
+      <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>select_one niveles_dano</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>dano_columnetas</t>
+          <t>dano_muros_portantes_pct</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1665,28 +1657,36 @@
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21')</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr"/>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21' or ${sistema_estructural} = '22' or ${sistema_estructural} = '23' or ${sistema_estructural} = '51' or ${sistema_estructural} = '52' or ${sistema_estructural} = '50' or ${sistema_estructural} = '60') and ${dano_muros_portantes} != 'ninguno'</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>. &gt;= 1 and . &lt;= 100</t>
+        </is>
+      </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Daño en columnetas de confinamiento</t>
+          <t>% de extensión del daño en muros portantes</t>
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Debe estar entre 1 y 100</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one niveles_dano</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>dano_columnetas_pct</t>
+          <t>dano_columnetas</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1697,36 +1697,28 @@
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21') and ${dano_columnetas} != 'ninguno'</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>. &gt;= 1 and . &lt;= 100</t>
-        </is>
-      </c>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21')</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>% de extensión del daño en columnetas de confinamiento</t>
+          <t>Daño en columnetas de confinamiento</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>Debe estar entre 1 y 100</t>
-        </is>
-      </c>
+      <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>select_one niveles_dano</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>dano_vigas_confinamiento</t>
+          <t>dano_columnetas_pct</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1737,28 +1729,36 @@
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21')</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr"/>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21') and ${dano_columnetas} != 'ninguno'</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>. &gt;= 1 and . &lt;= 100</t>
+        </is>
+      </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Daño en vigas de confinamiento</t>
+          <t>% de extensión del daño en columnetas de confinamiento</t>
         </is>
       </c>
       <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Debe estar entre 1 y 100</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one niveles_dano</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>dano_vigas_confinamiento_pct</t>
+          <t>dano_vigas_confinamiento</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1769,36 +1769,28 @@
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21') and ${dano_vigas_confinamiento} != 'ninguno'</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>. &gt;= 1 and . &lt;= 100</t>
-        </is>
-      </c>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21')</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
-          <t>% de extensión del daño en vigas de confinamiento</t>
+          <t>Daño en vigas de confinamiento</t>
         </is>
       </c>
       <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>Debe estar entre 1 y 100</t>
-        </is>
-      </c>
+      <c r="J41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>select_one niveles_dano</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>dano_entrepisos</t>
+          <t>dano_vigas_confinamiento_pct</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1809,28 +1801,36 @@
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42' or ${sistema_estructural} = '21' or ${sistema_estructural} = '22' or ${sistema_estructural} = '23' or ${sistema_estructural} = '51' or ${sistema_estructural} = '52' or ${sistema_estructural} = '50' or ${sistema_estructural} = '60')</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr"/>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21') and ${dano_vigas_confinamiento} != 'ninguno'</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>. &gt;= 1 and . &lt;= 100</t>
+        </is>
+      </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Daño en entrepisos</t>
+          <t>% de extensión del daño en vigas de confinamiento</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Debe estar entre 1 y 100</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one niveles_dano</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>dano_entrepisos_pct</t>
+          <t>dano_entrepisos</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1841,36 +1841,28 @@
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42' or ${sistema_estructural} = '21' or ${sistema_estructural} = '22' or ${sistema_estructural} = '23' or ${sistema_estructural} = '51' or ${sistema_estructural} = '52' or ${sistema_estructural} = '50' or ${sistema_estructural} = '60') and ${dano_entrepisos} != 'ninguno'</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>. &gt;= 1 and . &lt;= 100</t>
-        </is>
-      </c>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42' or ${sistema_estructural} = '21' or ${sistema_estructural} = '22' or ${sistema_estructural} = '23' or ${sistema_estructural} = '51' or ${sistema_estructural} = '52' or ${sistema_estructural} = '50' or ${sistema_estructural} = '60')</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
-          <t>% de extensión del daño en entrepisos</t>
+          <t>Daño en entrepisos</t>
         </is>
       </c>
       <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>Debe estar entre 1 y 100</t>
-        </is>
-      </c>
+      <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>select_multiple senales</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>senales_alarma</t>
+          <t>dano_entrepisos_pct</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1881,40 +1873,36 @@
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada'</t>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42' or ${sistema_estructural} = '21' or ${sistema_estructural} = '22' or ${sistema_estructural} = '23' or ${sistema_estructural} = '51' or ${sistema_estructural} = '52' or ${sistema_estructural} = '50' or ${sistema_estructural} = '60') and ${dano_entrepisos} != 'ninguno'</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>not(selected(., 'ninguna') and count-selected(.) &gt; 1)</t>
+          <t>. &gt;= 1 and . &lt;= 100</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Señales de alarma observadas</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>Marcar todas las que apliquen; si no hay, marcar «Ninguna»</t>
-        </is>
-      </c>
+          <t>% de extensión del daño en entrepisos</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr">
         <is>
-          <t>«Ninguna» no puede combinarse con otras señales</t>
+          <t>Debe estar entre 1 y 100</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>select_one danos_globales</t>
+          <t>select_multiple senales</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>dano_global</t>
+          <t>senales_alarma</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1928,25 +1916,37 @@
           <t>${tipo_inspeccion} != 'no_inspeccionada'</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>not(selected(., 'ninguna') and count-selected(.) &gt; 1)</t>
+        </is>
+      </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Porcentaje global de daño de la edificación</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
+          <t>Señales de alarma observadas</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Marcar todas las que apliquen; si no hay, marcar «Ninguna»</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>«Ninguna» no puede combinarse con otras señales</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>image</t>
+          <t>select_one danos_globales</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>foto_fachada</t>
+          <t>dano_global</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1955,23 +1955,19 @@
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>${tipo_inspeccion} != 'no_inspeccionada'</t>
+        </is>
+      </c>
       <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>max-pixels=1600</t>
-        </is>
-      </c>
+      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Foto: fachada completa</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>Desde el frente, que se vea todo el edificio</t>
-        </is>
-      </c>
+          <t>Porcentaje global de daño de la edificación</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr"/>
     </row>
     <row r="47">
@@ -1982,7 +1978,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>foto_esquina_1</t>
+          <t>foto_fachada</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2000,10 +1996,14 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Foto: esquina 1</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr"/>
+          <t>Foto: fachada completa</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Desde el frente, que se vea todo el edificio</t>
+        </is>
+      </c>
       <c r="J47" t="inlineStr"/>
     </row>
     <row r="48">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>foto_esquina_2</t>
+          <t>foto_esquina_1</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Foto: esquina 2</t>
+          <t>Foto: esquina 1</t>
         </is>
       </c>
       <c r="I48" t="inlineStr"/>
@@ -2046,10 +2046,14 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>foto_esquina_3</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr"/>
+          <t>foto_esquina_2</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr"/>
@@ -2060,7 +2064,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Foto: esquina 3 (si es accesible)</t>
+          <t>Foto: esquina 2</t>
         </is>
       </c>
       <c r="I49" t="inlineStr"/>
@@ -2074,7 +2078,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>foto_esquina_4</t>
+          <t>foto_esquina_3</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -2088,7 +2092,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Foto: esquina 4 (si es accesible)</t>
+          <t>Foto: esquina 3 (si es accesible)</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
@@ -2102,36 +2106,24 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>foto_grieta</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>foto_esquina_4</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada'</t>
-        </is>
-      </c>
+      <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>max-pixels=2048</t>
+          <t>max-pixels=1600</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Foto: peor grieta, de cerca</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>Poner una moneda junto a la grieta como referencia de escala</t>
-        </is>
-      </c>
+          <t>Foto: esquina 4 (si es accesible)</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr"/>
     </row>
     <row r="52">
@@ -2142,7 +2134,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>foto_columnas</t>
+          <t>foto_grieta</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2159,16 +2151,56 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
+          <t>max-pixels=2048</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Foto: peor grieta, de cerca</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Poner una moneda junto a la grieta como referencia de escala</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>foto_columnas</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>${tipo_inspeccion} != 'no_inspeccionada'</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
+        <is>
           <t>max-pixels=1600</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
+      <c r="H53" t="inlineStr">
         <is>
           <t>Foto: columnas del primer piso</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2181,7 +2213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C96"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2204,34 +2236,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>tipos_inspeccion</t>
+          <t>confirmaciones</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>exterior</t>
+          <t>si</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Solo exterior</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>tipos_inspeccion</t>
+          <t>confirmaciones</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>parcial</t>
+          <t>no_aplica</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Parcial (exterior + algunas zonas interiores)</t>
+          <t>No aplica (inmueble desocupado o sin acceso)</t>
         </is>
       </c>
     </row>
@@ -2243,12 +2275,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>completa</t>
+          <t>exterior</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Completa</t>
+          <t>Solo exterior</t>
         </is>
       </c>
     </row>
@@ -2260,46 +2292,46 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>no_inspeccionada</t>
+          <t>parcial</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>No se inspeccionó</t>
+          <t>Parcial (exterior + algunas zonas interiores)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>motivos_no_inspeccion</t>
+          <t>tipos_inspeccion</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>no_permitido</t>
+          <t>completa</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>No se permitió el acceso</t>
+          <t>Completa</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>motivos_no_inspeccion</t>
+          <t>tipos_inspeccion</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>desocupada</t>
+          <t>no_inspeccionada</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Edificación desocupada</t>
+          <t>No se inspeccionó</t>
         </is>
       </c>
     </row>
@@ -2311,12 +2343,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>colapso</t>
+          <t>no_permitido</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Colapso total</t>
+          <t>No se permitió el acceso</t>
         </is>
       </c>
     </row>
@@ -2328,12 +2360,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>demolida</t>
+          <t>desocupada</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Ya demolida</t>
+          <t>Edificación desocupada</t>
         </is>
       </c>
     </row>
@@ -2345,46 +2377,46 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>otro</t>
+          <t>colapso</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Otro</t>
+          <t>Colapso total</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>comunas</t>
+          <t>motivos_no_inspeccion</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>centro</t>
+          <t>demolida</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Centro</t>
+          <t>Ya demolida</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>comunas</t>
+          <t>motivos_no_inspeccion</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>rio_otun</t>
+          <t>otro</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Río Otún</t>
+          <t>Otro</t>
         </is>
       </c>
     </row>
@@ -2396,12 +2428,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>villavicencio</t>
+          <t>centro</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Villavicencio</t>
+          <t>Centro</t>
         </is>
       </c>
     </row>
@@ -2413,12 +2445,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>villa_santana</t>
+          <t>rio_otun</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Villa Santana</t>
+          <t>Río Otún</t>
         </is>
       </c>
     </row>
@@ -2430,12 +2462,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>oriente</t>
+          <t>villavicencio</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Oriente</t>
+          <t>Villavicencio</t>
         </is>
       </c>
     </row>
@@ -2447,12 +2479,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>universidad</t>
+          <t>villa_santana</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Universidad</t>
+          <t>Villa Santana</t>
         </is>
       </c>
     </row>
@@ -2464,12 +2496,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>boston</t>
+          <t>oriente</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Oriente</t>
         </is>
       </c>
     </row>
@@ -2481,12 +2513,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>jardin</t>
+          <t>universidad</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Jardín</t>
+          <t>Universidad</t>
         </is>
       </c>
     </row>
@@ -2498,12 +2530,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>cuba</t>
+          <t>boston</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Cuba</t>
+          <t>Boston</t>
         </is>
       </c>
     </row>
@@ -2515,12 +2547,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>consota</t>
+          <t>jardin</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Consotá</t>
+          <t>Jardín</t>
         </is>
       </c>
     </row>
@@ -2532,12 +2564,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>el_oso</t>
+          <t>cuba</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>El Oso</t>
+          <t>Cuba</t>
         </is>
       </c>
     </row>
@@ -2549,12 +2581,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>san_joaquin</t>
+          <t>consota</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>San Joaquín</t>
+          <t>Consotá</t>
         </is>
       </c>
     </row>
@@ -2566,12 +2598,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>perla_del_otun</t>
+          <t>el_oso</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Perla del Otún</t>
+          <t>El Oso</t>
         </is>
       </c>
     </row>
@@ -2583,12 +2615,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>olimpica</t>
+          <t>san_joaquin</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Olímpica</t>
+          <t>San Joaquín</t>
         </is>
       </c>
     </row>
@@ -2600,12 +2632,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ferrocarril</t>
+          <t>perla_del_otun</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Ferrocarril</t>
+          <t>Perla del Otún</t>
         </is>
       </c>
     </row>
@@ -2617,12 +2649,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>del_cafe</t>
+          <t>olimpica</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Del Café</t>
+          <t>Olímpica</t>
         </is>
       </c>
     </row>
@@ -2634,12 +2666,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>el_poblado</t>
+          <t>ferrocarril</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>El Poblado</t>
+          <t>Ferrocarril</t>
         </is>
       </c>
     </row>
@@ -2651,12 +2683,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>el_rocio</t>
+          <t>del_cafe</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>El Rocío</t>
+          <t>Del Café</t>
         </is>
       </c>
     </row>
@@ -2668,12 +2700,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>san_nicolas</t>
+          <t>el_poblado</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>San Nicolás</t>
+          <t>El Poblado</t>
         </is>
       </c>
     </row>
@@ -2685,46 +2717,46 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>otro</t>
+          <t>el_rocio</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Otra / zona rural</t>
+          <t>El Rocío</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>sistemas_estructurales</t>
+          <t>comunas</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>san_nicolas</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Concreto: pórtico</t>
+          <t>San Nicolás</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>sistemas_estructurales</t>
+          <t>comunas</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>otro</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Concreto: muros estructurales</t>
+          <t>Otra / zona rural</t>
         </is>
       </c>
     </row>
@@ -2736,12 +2768,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Concreto: sistema dual (pórtico + muros)</t>
+          <t>Concreto: pórtico</t>
         </is>
       </c>
     </row>
@@ -2753,12 +2785,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Concreto: prefabricado</t>
+          <t>Concreto: muros estructurales</t>
         </is>
       </c>
     </row>
@@ -2770,12 +2802,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Mampostería confinada (con vigas y columnas de amarre)</t>
+          <t>Concreto: sistema dual (pórtico + muros)</t>
         </is>
       </c>
     </row>
@@ -2787,12 +2819,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Mampostería reforzada</t>
+          <t>Concreto: prefabricado</t>
         </is>
       </c>
     </row>
@@ -2804,12 +2836,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Mampostería no reforzada (sin amarres)</t>
+          <t>Mampostería confinada (con vigas y columnas de amarre)</t>
         </is>
       </c>
     </row>
@@ -2821,12 +2853,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Acero: pórticos arriostrados</t>
+          <t>Mampostería reforzada</t>
         </is>
       </c>
     </row>
@@ -2838,12 +2870,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>23</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Acero: pórticos no arriostrados</t>
+          <t>Mampostería no reforzada (sin amarres)</t>
         </is>
       </c>
     </row>
@@ -2855,12 +2887,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>31</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Acero: pórticos en celosía</t>
+          <t>Acero: pórticos arriostrados</t>
         </is>
       </c>
     </row>
@@ -2872,12 +2904,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>32</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Madera: pórticos y panel en madera</t>
+          <t>Acero: pórticos no arriostrados</t>
         </is>
       </c>
     </row>
@@ -2889,12 +2921,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>33</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Madera: pórticos con paneles de otros materiales</t>
+          <t>Acero: pórticos en celosía</t>
         </is>
       </c>
     </row>
@@ -2906,12 +2938,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>41</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Muros en bahareque</t>
+          <t>Madera: pórticos y panel en madera</t>
         </is>
       </c>
     </row>
@@ -2923,12 +2955,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>42</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Muros en tapia</t>
+          <t>Madera: pórticos con paneles de otros materiales</t>
         </is>
       </c>
     </row>
@@ -2940,12 +2972,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>51</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Mixta</t>
+          <t>Muros en bahareque</t>
         </is>
       </c>
     </row>
@@ -2957,46 +2989,46 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>52</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Otros / no identificable</t>
+          <t>Muros en tapia</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>tipos_entrepiso</t>
+          <t>sistemas_estructurales</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>50</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Concreto: placa maciza</t>
+          <t>Mixta</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>tipos_entrepiso</t>
+          <t>sistemas_estructurales</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Concreto: placa aligerada</t>
+          <t>Otros / no identificable</t>
         </is>
       </c>
     </row>
@@ -3008,12 +3040,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Concreto: reticular celulado</t>
+          <t>Concreto: placa maciza</t>
         </is>
       </c>
     </row>
@@ -3025,12 +3057,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Acero: vigas alma llena con conectores</t>
+          <t>Concreto: placa aligerada</t>
         </is>
       </c>
     </row>
@@ -3042,12 +3074,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Acero: vigas alma llena sin conectores</t>
+          <t>Concreto: reticular celulado</t>
         </is>
       </c>
     </row>
@@ -3059,12 +3091,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Acero: cerchas</t>
+          <t>Acero: vigas alma llena con conectores</t>
         </is>
       </c>
     </row>
@@ -3076,12 +3108,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Madera: vigas</t>
+          <t>Acero: vigas alma llena sin conectores</t>
         </is>
       </c>
     </row>
@@ -3093,12 +3125,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>23</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Madera: cerchas</t>
+          <t>Acero: cerchas</t>
         </is>
       </c>
     </row>
@@ -3110,12 +3142,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>31</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Mixta</t>
+          <t>Madera: vigas</t>
         </is>
       </c>
     </row>
@@ -3127,46 +3159,46 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>32</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Otros / no se sabe</t>
+          <t>Madera: cerchas</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>usos</t>
+          <t>tipos_entrepiso</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>40</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Residencial</t>
+          <t>Mixta</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>usos</t>
+          <t>tipos_entrepiso</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>50</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Comercial</t>
+          <t>Otros / no se sabe</t>
         </is>
       </c>
     </row>
@@ -3178,12 +3210,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Educacional</t>
+          <t>Residencial</t>
         </is>
       </c>
     </row>
@@ -3195,12 +3227,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Comercial</t>
         </is>
       </c>
     </row>
@@ -3212,12 +3244,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Hotelero</t>
+          <t>Educacional</t>
         </is>
       </c>
     </row>
@@ -3229,12 +3261,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Oficinas</t>
+          <t>Salud</t>
         </is>
       </c>
     </row>
@@ -3246,12 +3278,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Hotelero</t>
         </is>
       </c>
     </row>
@@ -3263,12 +3295,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Institucional</t>
+          <t>Oficinas</t>
         </is>
       </c>
     </row>
@@ -3280,12 +3312,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Bodegas</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -3297,12 +3329,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Estacionamientos</t>
+          <t>Institucional</t>
         </is>
       </c>
     </row>
@@ -3314,46 +3346,46 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Otros</t>
+          <t>Bodegas</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>rangos_ano</t>
+          <t>usos</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Antes de 1950</t>
+          <t>Estacionamientos</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>rangos_ano</t>
+          <t>usos</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>1950 – 1982</t>
+          <t>Otros</t>
         </is>
       </c>
     </row>
@@ -3365,12 +3397,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>1982 – 1997</t>
+          <t>Antes de 1950</t>
         </is>
       </c>
     </row>
@@ -3382,46 +3414,46 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>1998 en adelante</t>
+          <t>1950 – 1982</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>colapsos</t>
+          <t>rangos_ano</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Colapso total</t>
+          <t>1982 – 1997</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>colapsos</t>
+          <t>rangos_ano</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>parcial_mayor_50</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Colapso parcial (50% o más)</t>
+          <t>1998 en adelante</t>
         </is>
       </c>
     </row>
@@ -3433,12 +3465,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>parcial_menor_50</t>
+          <t>total</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Colapso parcial (menos del 50%)</t>
+          <t>Colapso total</t>
         </is>
       </c>
     </row>
@@ -3450,46 +3482,46 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>ninguno</t>
+          <t>parcial_mayor_50</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>Colapso parcial (50% o más)</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>inclinaciones</t>
+          <t>colapsos</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>evidente</t>
+          <t>parcial_menor_50</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Inclinación evidente</t>
+          <t>Colapso parcial (menos del 50%)</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>inclinaciones</t>
+          <t>colapsos</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>dudas</t>
+          <t>ninguno</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Hay dudas</t>
+          <t>Ninguno</t>
         </is>
       </c>
     </row>
@@ -3501,46 +3533,46 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ninguna</t>
+          <t>evidente</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Inclinación evidente</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>niveles_dano</t>
+          <t>inclinaciones</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>ninguno</t>
+          <t>dudas</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Ninguno / muy leve</t>
+          <t>Hay dudas</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>niveles_dano</t>
+          <t>inclinaciones</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>leve</t>
+          <t>ninguna</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Leve</t>
+          <t>Ninguna</t>
         </is>
       </c>
     </row>
@@ -3552,12 +3584,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>moderado</t>
+          <t>ninguno</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Ninguno / muy leve</t>
         </is>
       </c>
     </row>
@@ -3569,12 +3601,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>fuerte</t>
+          <t>leve</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Fuerte</t>
+          <t>Leve</t>
         </is>
       </c>
     </row>
@@ -3586,46 +3618,46 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>severo</t>
+          <t>moderado</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Severo</t>
+          <t>Moderado</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>danos_globales</t>
+          <t>niveles_dano</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>ninguno</t>
+          <t>fuerte</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>Fuerte</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>danos_globales</t>
+          <t>niveles_dano</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>0_10</t>
+          <t>severo</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0 – 10 %</t>
+          <t>Severo</t>
         </is>
       </c>
     </row>
@@ -3637,12 +3669,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>10_30</t>
+          <t>ninguno</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>10 – 30 %</t>
+          <t>Ninguno</t>
         </is>
       </c>
     </row>
@@ -3654,12 +3686,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>30_60</t>
+          <t>0_10</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>30 – 60 %</t>
+          <t>0 – 10 %</t>
         </is>
       </c>
     </row>
@@ -3671,12 +3703,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>60_100</t>
+          <t>10_30</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>60 – 100 %</t>
+          <t>10 – 30 %</t>
         </is>
       </c>
     </row>
@@ -3688,46 +3720,46 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>30_60</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>100 % (colapso)</t>
+          <t>30 – 60 %</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>senales</t>
+          <t>danos_globales</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>grietas_x</t>
+          <t>60_100</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Grietas en X en muros</t>
+          <t>60 – 100 %</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>senales</t>
+          <t>danos_globales</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>grietas_horizontales_base</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Grietas horizontales en base de columnas</t>
+          <t>100 % (colapso)</t>
         </is>
       </c>
     </row>
@@ -3739,12 +3771,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>refuerzo_expuesto</t>
+          <t>grietas_x</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Refuerzo (varillas) expuesto</t>
+          <t>Grietas en X en muros</t>
         </is>
       </c>
     </row>
@@ -3756,12 +3788,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>pisos_desnivelados</t>
+          <t>grietas_horizontales_base</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Pisos desnivelados o inclinados</t>
+          <t>Grietas horizontales en base de columnas</t>
         </is>
       </c>
     </row>
@@ -3773,12 +3805,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>separacion_muro_estructura</t>
+          <t>refuerzo_expuesto</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Separación entre muros y estructura</t>
+          <t>Refuerzo (varillas) expuesto</t>
         </is>
       </c>
     </row>
@@ -3790,12 +3822,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>grieta_ancha</t>
+          <t>pisos_desnivelados</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Grieta llamativamente ancha (fotografiar con escala)</t>
+          <t>Pisos desnivelados o inclinados</t>
         </is>
       </c>
     </row>
@@ -3807,10 +3839,44 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
+          <t>separacion_muro_estructura</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Separación entre muros y estructura</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>senales</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>grieta_ancha</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Grieta llamativamente ancha (fotografiar con escala)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>senales</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
           <t>ninguna</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
+      <c r="C98" t="inlineStr">
         <is>
           <t>Ninguna</t>
         </is>
@@ -3865,7 +3931,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026081603</t>
+          <t>2026081604</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">

</xml_diff>

<commit_message>
Arreglar choice_filter de barrio: Enketo no soporta if() en el filtro
Enketo fallaba al cargar el formulario con FormLogicError "Too many
tokens" porque el choice_filter de barrio anidaba un if() dentro del
predicado. Su evaluador de filtros solo acepta comparaciones planas
unidas por and/or, así que la división efectiva (comuna o corregimiento
según tipo_zona) se resuelve ahora en un calculate (division_sel) y el
filtro queda plano: division_code=${division_sel} or name='OTRO'.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/kobo/ais.xlsx
+++ b/kobo/ais.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:M66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,15 +466,20 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>calculation</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>label::Español (es)</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>hint::Español (es)</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>constraint_message::Español (es)</t>
         </is>
@@ -501,6 +506,7 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -523,6 +529,7 @@
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -545,6 +552,7 @@
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -564,13 +572,14 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr">
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
         <is>
           <t>AVISO DE PRIVACIDAD — Esta inspección registra ubicación, características y fotografías de la edificación (solo exteriores y elementos estructurales, no personas ni interiores habitados salvo lo estrictamente necesario) para priorizar la evaluación estructural post-sismo. Tratamiento según la Ley 1581 de 2012; política completa disponible con la entidad coordinadora. La clasificación resultante es un insumo de priorización: la habilitación definitiva es competencia de las autoridades.</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -594,17 +603,18 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr">
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
         <is>
           <t>¿Informaste al ocupante o responsable del inmueble el propósito de la inspección y el aviso de privacidad?</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>Si no hay nadie presente, marca «No aplica (inmueble desocupado o sin acceso)»</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -628,13 +638,14 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr">
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
         <is>
           <t>Tipo de inspección</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -662,13 +673,14 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr">
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
         <is>
           <t>¿Por qué no se inspeccionó?</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -696,13 +708,14 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr">
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
         <is>
           <t>Municipio</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -726,13 +739,14 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr">
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
         <is>
           <t>Tipo de zona</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -768,13 +782,14 @@
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr">
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
         <is>
           <t>Comuna</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -810,61 +825,51 @@
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr">
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
         <is>
           <t>Corregimiento</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>select_one_from_file barrios.csv</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>barrio</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>minimal</t>
-        </is>
-      </c>
+          <t>division_sel</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>division_code=if(${tipo_zona} = 'urbano', ${division_urbana}, ${division_rural}) or name='OTRO'</t>
-        </is>
-      </c>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Barrio / Vereda</t>
+          <t>if(${tipo_zona} = 'urbano', ${division_urbana}, ${division_rural})</t>
         </is>
       </c>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one_from_file barrios.csv</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>barrio_otro</t>
+          <t>barrio</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -872,63 +877,73 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>${barrio} = 'OTRO'</t>
-        </is>
-      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>minimal</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>division_code=${division_sel} or name='OTRO'</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>¿Cuál?</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Barrio / Vereda</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>select_one via_tipo</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>via_tipo</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
+          <t>barrio_otro</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>${tipo_zona} = 'urbano'</t>
+          <t>${barrio} = 'OTRO'</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Tipo de vía</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>¿Cuál?</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one via_tipo</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>via_numero</t>
+          <t>via_tipo</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -942,13 +957,14 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Número de vía</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Tipo de vía</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -958,7 +974,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>numero_placa</t>
+          <t>via_numero</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -972,13 +988,14 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>Número (placa)</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Número de vía</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -988,27 +1005,28 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>referencia_ubicacion</t>
+          <t>numero_placa</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>${tipo_zona} = 'urbano'</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>Referencia de ubicación</t>
-        </is>
-      </c>
+      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Finca, kilómetro, punto de referencia</t>
+          <t>Número (placa)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1018,7 +1036,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>nombre_edificacion</t>
+          <t>referencia_ubicacion</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -1028,111 +1046,119 @@
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>Nombre de la edificación (si tiene)</t>
-        </is>
-      </c>
+      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Propiedad horizontal o institución</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr"/>
+          <t>Referencia de ubicación</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Finca, kilómetro, punto de referencia</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>geopoint</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ubicacion</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>nombre_edificacion</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>Ubicación GPS</t>
-        </is>
-      </c>
+      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Capturar de pie frente a la edificación, con cielo visible. Si no captura bajo techo, reintentar afuera.</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr"/>
+          <t>Nombre de la edificación (si tiene)</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Propiedad horizontal o institución</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>geopoint</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>catastral</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>field-list</t>
-        </is>
-      </c>
+          <t>ubicacion</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>Identificación catastral (opcional)</t>
-        </is>
-      </c>
+      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Solo si tiene el recibo de predial a la vista</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr"/>
+          <t>Ubicación GPS</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Capturar de pie frente a la edificación, con cielo visible. Si no captura bajo techo, reintentar afuera.</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>cat_sector</t>
+          <t>catastral</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>Sector</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Identificación catastral (opcional)</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Solo si tiene el recibo de predial a la vista</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1142,7 +1168,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>cat_manzana</t>
+          <t>cat_sector</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1152,13 +1178,14 @@
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>Manzana</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1168,7 +1195,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>cat_predio</t>
+          <t>cat_manzana</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1178,13 +1205,14 @@
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>Predio</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Manzana</t>
+        </is>
+      </c>
       <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1194,7 +1222,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>cat_mejora</t>
+          <t>cat_predio</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1204,21 +1232,26 @@
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>Mejora / Prop. horizontal</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Predio</t>
+        </is>
+      </c>
       <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>cat_mejora</t>
+        </is>
+      </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr"/>
@@ -1227,50 +1260,32 @@
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Mejora / Prop. horizontal</t>
+        </is>
+      </c>
       <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>pisos_sobre</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada'</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>. &gt;= 1 and . &lt;= 50</t>
-        </is>
-      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>Niveles sobre el terreno</t>
-        </is>
-      </c>
+      <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>Debe estar entre 1 y 50</t>
-        </is>
-      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1280,10 +1295,14 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>sotanos</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr"/>
+          <t>pisos_sobre</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
@@ -1292,61 +1311,63 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>. &gt;= 0 and . &lt;= 10</t>
+          <t>. &gt;= 1 and . &lt;= 50</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>Sótanos</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>Debe estar entre 0 y 10</t>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Niveles sobre el terreno</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Debe estar entre 1 y 50</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>select_one usos</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>uso_predominante</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>minimal</t>
-        </is>
-      </c>
+          <t>sotanos</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>${tipo_inspeccion} != 'no_inspeccionada'</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 10</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>Uso predominante de la edificación</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Sótanos</t>
+        </is>
+      </c>
       <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Debe estar entre 0 y 10</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1356,10 +1377,14 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>uso_planta_baja</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr"/>
+          <t>uso_predominante</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="D30" t="inlineStr">
         <is>
           <t>minimal</t>
@@ -1374,51 +1399,49 @@
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>Uso de la planta baja</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Uso predominante de la edificación</t>
+        </is>
+      </c>
       <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>select_one usos</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>frente_m</t>
+          <t>uso_planta_baja</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>minimal</t>
+        </is>
+      </c>
       <c r="E31" t="inlineStr">
         <is>
           <t>${tipo_inspeccion} != 'no_inspeccionada'</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>. &gt; 0 and . &lt; 1000</t>
-        </is>
-      </c>
+      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>Frente aproximado (m)</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>Valor en metros, mayor que 0</t>
-        </is>
-      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Uso de la planta baja</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1428,7 +1451,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>fondo_m</t>
+          <t>frente_m</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -1446,13 +1469,14 @@
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>Fondo aproximado (m)</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr">
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Frente aproximado (m)</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr">
         <is>
           <t>Valor en metros, mayor que 0</t>
         </is>
@@ -1461,53 +1485,58 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>select_one sistemas_estructurales</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>sistema_estructural</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>minimal</t>
-        </is>
-      </c>
+          <t>fondo_m</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>${tipo_inspeccion} != 'no_inspeccionada'</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>. &gt; 0 and . &lt; 1000</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>Sistema estructural</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Fondo aproximado (m)</t>
+        </is>
+      </c>
       <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Valor en metros, mayor que 0</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>select_one tipos_entrepiso</t>
+          <t>select_one sistemas_estructurales</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>tipo_entrepiso</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr"/>
+          <t>sistema_estructural</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
           <t>minimal</t>
@@ -1522,31 +1551,32 @@
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>Tipo de entrepiso</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Sistema estructural</t>
+        </is>
+      </c>
       <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>select_one rangos_ano</t>
+          <t>select_one tipos_entrepiso</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>rango_ano</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr"/>
+          <t>tipo_entrepiso</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>minimal</t>
+        </is>
+      </c>
       <c r="E35" t="inlineStr">
         <is>
           <t>${tipo_inspeccion} != 'no_inspeccionada'</t>
@@ -1556,23 +1586,24 @@
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>Año de construcción</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Tipo de entrepiso</t>
+        </is>
+      </c>
       <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>select_one colapsos</t>
+          <t>select_one rangos_ano</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>colapso</t>
+          <t>rango_ano</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1590,23 +1621,24 @@
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>Colapso</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Año de construcción</t>
+        </is>
+      </c>
       <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>select_one inclinaciones</t>
+          <t>select_one colapsos</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>inclinacion</t>
+          <t>colapso</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1624,23 +1656,24 @@
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>Inclinación de la edificación o de un piso</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Colapso</t>
+        </is>
+      </c>
       <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one inclinaciones</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>piso_mayor_dano</t>
+          <t>inclinacion</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1651,42 +1684,31 @@
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and ${colapso} != 'total'</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>. &gt;= 0 and . &lt;= 50</t>
-        </is>
-      </c>
+          <t>${tipo_inspeccion} != 'no_inspeccionada'</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>¿Cuál es el piso de mayor daño?</t>
-        </is>
-      </c>
+      <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
-          <t>La matriz de daño se evalúa en ese piso</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>0 = sótano; máximo 50</t>
-        </is>
-      </c>
+          <t>Inclinación de la edificación o de un piso</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>select_one niveles_dano</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>dano_vigas</t>
+          <t>piso_mayor_dano</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1697,30 +1719,43 @@
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42')</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr"/>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and ${colapso} != 'total'</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 50</t>
+        </is>
+      </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>Daño en vigas</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>¿Cuál es el piso de mayor daño?</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>La matriz de daño se evalúa en ese piso</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>0 = sótano; máximo 50</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one niveles_dano</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>dano_vigas_pct</t>
+          <t>dano_vigas</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1731,38 +1766,31 @@
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42') and ${dano_vigas} != 'ninguno'</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>. &gt;= 1 and . &lt;= 100</t>
-        </is>
-      </c>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42')</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>% de extensión del daño en vigas</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>Debe estar entre 1 y 100</t>
-        </is>
-      </c>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Daño en vigas</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>select_one niveles_dano</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>dano_columnas</t>
+          <t>dano_vigas_pct</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1773,30 +1801,39 @@
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42')</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr"/>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42') and ${dano_vigas} != 'ninguno'</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>. &gt;= 1 and . &lt;= 100</t>
+        </is>
+      </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>Daño en columnas</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>% de extensión del daño en vigas</t>
+        </is>
+      </c>
       <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Debe estar entre 1 y 100</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one niveles_dano</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>dano_columnas_pct</t>
+          <t>dano_columnas</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1807,38 +1844,31 @@
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42') and ${dano_columnas} != 'ninguno'</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>. &gt;= 1 and . &lt;= 100</t>
-        </is>
-      </c>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42')</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>% de extensión del daño en columnas</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>Debe estar entre 1 y 100</t>
-        </is>
-      </c>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Daño en columnas</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>select_one niveles_dano</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>dano_nudos</t>
+          <t>dano_columnas_pct</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1849,30 +1879,39 @@
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14')</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr"/>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42') and ${dano_columnas} != 'ninguno'</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>. &gt;= 1 and . &lt;= 100</t>
+        </is>
+      </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>Daño en nudos (unión viga-columna)</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>% de extensión del daño en columnas</t>
+        </is>
+      </c>
       <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>Debe estar entre 1 y 100</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one niveles_dano</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>dano_nudos_pct</t>
+          <t>dano_nudos</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1883,38 +1922,31 @@
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14') and ${dano_nudos} != 'ninguno'</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>. &gt;= 1 and . &lt;= 100</t>
-        </is>
-      </c>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14')</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>% de extensión del daño en nudos (unión viga-columna)</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>Debe estar entre 1 y 100</t>
-        </is>
-      </c>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Daño en nudos (unión viga-columna)</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>select_one niveles_dano</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>dano_conexiones</t>
+          <t>dano_nudos_pct</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1925,30 +1957,39 @@
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42')</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr"/>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14') and ${dano_nudos} != 'ninguno'</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>. &gt;= 1 and . &lt;= 100</t>
+        </is>
+      </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>Daño en conexiones</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>% de extensión del daño en nudos (unión viga-columna)</t>
+        </is>
+      </c>
       <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>Debe estar entre 1 y 100</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one niveles_dano</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>dano_conexiones_pct</t>
+          <t>dano_conexiones</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1959,38 +2000,31 @@
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42') and ${dano_conexiones} != 'ninguno'</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>. &gt;= 1 and . &lt;= 100</t>
-        </is>
-      </c>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42')</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>% de extensión del daño en conexiones</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>Debe estar entre 1 y 100</t>
-        </is>
-      </c>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Daño en conexiones</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>select_one niveles_dano</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>dano_muros</t>
+          <t>dano_conexiones_pct</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2001,30 +2035,39 @@
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '12' or ${sistema_estructural} = '13')</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr"/>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42') and ${dano_conexiones} != 'ninguno'</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>. &gt;= 1 and . &lt;= 100</t>
+        </is>
+      </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>Daño en muros estructurales</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>% de extensión del daño en conexiones</t>
+        </is>
+      </c>
       <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>Debe estar entre 1 y 100</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one niveles_dano</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>dano_muros_pct</t>
+          <t>dano_muros</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2035,38 +2078,31 @@
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '12' or ${sistema_estructural} = '13') and ${dano_muros} != 'ninguno'</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>. &gt;= 1 and . &lt;= 100</t>
-        </is>
-      </c>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '12' or ${sistema_estructural} = '13')</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>% de extensión del daño en muros estructurales</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>Debe estar entre 1 y 100</t>
-        </is>
-      </c>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Daño en muros estructurales</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>select_one niveles_dano</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>dano_muros_portantes</t>
+          <t>dano_muros_pct</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2077,30 +2113,39 @@
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21' or ${sistema_estructural} = '22' or ${sistema_estructural} = '23' or ${sistema_estructural} = '51' or ${sistema_estructural} = '52' or ${sistema_estructural} = '50' or ${sistema_estructural} = '60')</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr"/>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '12' or ${sistema_estructural} = '13') and ${dano_muros} != 'ninguno'</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>. &gt;= 1 and . &lt;= 100</t>
+        </is>
+      </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>Daño en muros portantes</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>% de extensión del daño en muros estructurales</t>
+        </is>
+      </c>
       <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>Debe estar entre 1 y 100</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one niveles_dano</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>dano_muros_portantes_pct</t>
+          <t>dano_muros_portantes</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2111,38 +2156,31 @@
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21' or ${sistema_estructural} = '22' or ${sistema_estructural} = '23' or ${sistema_estructural} = '51' or ${sistema_estructural} = '52' or ${sistema_estructural} = '50' or ${sistema_estructural} = '60') and ${dano_muros_portantes} != 'ninguno'</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>. &gt;= 1 and . &lt;= 100</t>
-        </is>
-      </c>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21' or ${sistema_estructural} = '22' or ${sistema_estructural} = '23' or ${sistema_estructural} = '51' or ${sistema_estructural} = '52' or ${sistema_estructural} = '50' or ${sistema_estructural} = '60')</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>% de extensión del daño en muros portantes</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>Debe estar entre 1 y 100</t>
-        </is>
-      </c>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Daño en muros portantes</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>select_one niveles_dano</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>dano_columnetas</t>
+          <t>dano_muros_portantes_pct</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2153,30 +2191,39 @@
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21')</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr"/>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21' or ${sistema_estructural} = '22' or ${sistema_estructural} = '23' or ${sistema_estructural} = '51' or ${sistema_estructural} = '52' or ${sistema_estructural} = '50' or ${sistema_estructural} = '60') and ${dano_muros_portantes} != 'ninguno'</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>. &gt;= 1 and . &lt;= 100</t>
+        </is>
+      </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>Daño en columnetas de confinamiento</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>% de extensión del daño en muros portantes</t>
+        </is>
+      </c>
       <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>Debe estar entre 1 y 100</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one niveles_dano</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>dano_columnetas_pct</t>
+          <t>dano_columnetas</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2187,38 +2234,31 @@
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21') and ${dano_columnetas} != 'ninguno'</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>. &gt;= 1 and . &lt;= 100</t>
-        </is>
-      </c>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21')</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>% de extensión del daño en columnetas de confinamiento</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>Debe estar entre 1 y 100</t>
-        </is>
-      </c>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Daño en columnetas de confinamiento</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>select_one niveles_dano</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>dano_vigas_confinamiento</t>
+          <t>dano_columnetas_pct</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2229,30 +2269,39 @@
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21')</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr"/>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21') and ${dano_columnetas} != 'ninguno'</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>. &gt;= 1 and . &lt;= 100</t>
+        </is>
+      </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>Daño en vigas de confinamiento</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>% de extensión del daño en columnetas de confinamiento</t>
+        </is>
+      </c>
       <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>Debe estar entre 1 y 100</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one niveles_dano</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>dano_vigas_confinamiento_pct</t>
+          <t>dano_vigas_confinamiento</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2263,38 +2312,31 @@
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21') and ${dano_vigas_confinamiento} != 'ninguno'</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>. &gt;= 1 and . &lt;= 100</t>
-        </is>
-      </c>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21')</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>% de extensión del daño en vigas de confinamiento</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>Debe estar entre 1 y 100</t>
-        </is>
-      </c>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Daño en vigas de confinamiento</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>select_one niveles_dano</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>dano_entrepisos</t>
+          <t>dano_vigas_confinamiento_pct</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2305,30 +2347,39 @@
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42' or ${sistema_estructural} = '21' or ${sistema_estructural} = '22' or ${sistema_estructural} = '23' or ${sistema_estructural} = '51' or ${sistema_estructural} = '52' or ${sistema_estructural} = '50' or ${sistema_estructural} = '60')</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr"/>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '21') and ${dano_vigas_confinamiento} != 'ninguno'</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>. &gt;= 1 and . &lt;= 100</t>
+        </is>
+      </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>Daño en entrepisos</t>
-        </is>
-      </c>
-      <c r="K55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>% de extensión del daño en vigas de confinamiento</t>
+        </is>
+      </c>
       <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>Debe estar entre 1 y 100</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one niveles_dano</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>dano_entrepisos_pct</t>
+          <t>dano_entrepisos</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2339,38 +2390,31 @@
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42' or ${sistema_estructural} = '21' or ${sistema_estructural} = '22' or ${sistema_estructural} = '23' or ${sistema_estructural} = '51' or ${sistema_estructural} = '52' or ${sistema_estructural} = '50' or ${sistema_estructural} = '60') and ${dano_entrepisos} != 'ninguno'</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>. &gt;= 1 and . &lt;= 100</t>
-        </is>
-      </c>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42' or ${sistema_estructural} = '21' or ${sistema_estructural} = '22' or ${sistema_estructural} = '23' or ${sistema_estructural} = '51' or ${sistema_estructural} = '52' or ${sistema_estructural} = '50' or ${sistema_estructural} = '60')</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>% de extensión del daño en entrepisos</t>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>Debe estar entre 1 y 100</t>
-        </is>
-      </c>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Daño en entrepisos</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>select_multiple senales</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>senales_alarma</t>
+          <t>dano_entrepisos_pct</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2381,42 +2425,39 @@
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada'</t>
+          <t>${tipo_inspeccion} != 'no_inspeccionada' and (${sistema_estructural} = '11' or ${sistema_estructural} = '12' or ${sistema_estructural} = '13' or ${sistema_estructural} = '14' or ${sistema_estructural} = '31' or ${sistema_estructural} = '32' or ${sistema_estructural} = '33' or ${sistema_estructural} = '41' or ${sistema_estructural} = '42' or ${sistema_estructural} = '21' or ${sistema_estructural} = '22' or ${sistema_estructural} = '23' or ${sistema_estructural} = '51' or ${sistema_estructural} = '52' or ${sistema_estructural} = '50' or ${sistema_estructural} = '60') and ${dano_entrepisos} != 'ninguno'</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>not(selected(., 'ninguna') and count-selected(.) &gt; 1)</t>
+          <t>. &gt;= 1 and . &lt;= 100</t>
         </is>
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>Señales de alarma observadas</t>
-        </is>
-      </c>
+      <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr">
         <is>
-          <t>Marcar todas las que apliquen; si no hay, marcar «Ninguna»</t>
-        </is>
-      </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>«Ninguna» no puede combinarse con otras señales</t>
+          <t>% de extensión del daño en entrepisos</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>Debe estar entre 1 y 100</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>select_one danos_globales</t>
+          <t>select_multiple senales</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>dano_global</t>
+          <t>senales_alarma</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2430,27 +2471,40 @@
           <t>${tipo_inspeccion} != 'no_inspeccionada'</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>not(selected(., 'ninguna') and count-selected(.) &gt; 1)</t>
+        </is>
+      </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>Porcentaje global de daño de la edificación</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Señales de alarma observadas</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Marcar todas las que apliquen; si no hay, marcar «Ninguna»</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>«Ninguna» no puede combinarse con otras señales</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>image</t>
+          <t>select_one danos_globales</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>foto_fachada</t>
+          <t>dano_global</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2459,26 +2513,23 @@
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>${tipo_inspeccion} != 'no_inspeccionada'</t>
+        </is>
+      </c>
       <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>max-pixels=1600</t>
-        </is>
-      </c>
+      <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>Foto: fachada completa</t>
-        </is>
-      </c>
+      <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr">
         <is>
-          <t>Desde el frente, que se vea todo el edificio</t>
+          <t>Porcentaje global de daño de la edificación</t>
         </is>
       </c>
       <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2488,7 +2539,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>foto_esquina_1</t>
+          <t>foto_fachada</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2506,13 +2557,18 @@
       </c>
       <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>Foto: esquina 1</t>
-        </is>
-      </c>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Foto: fachada completa</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Desde el frente, que se vea todo el edificio</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2522,7 +2578,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>foto_esquina_2</t>
+          <t>foto_esquina_1</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2540,13 +2596,14 @@
       </c>
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>Foto: esquina 2</t>
-        </is>
-      </c>
-      <c r="K61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Foto: esquina 1</t>
+        </is>
+      </c>
       <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2556,10 +2613,14 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>foto_esquina_3</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr"/>
+          <t>foto_esquina_2</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr"/>
@@ -2570,13 +2631,14 @@
       </c>
       <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>Foto: esquina 3 (si es accesible)</t>
-        </is>
-      </c>
-      <c r="K62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Foto: esquina 2</t>
+        </is>
+      </c>
       <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2586,7 +2648,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>foto_esquina_4</t>
+          <t>foto_esquina_3</t>
         </is>
       </c>
       <c r="C63" t="inlineStr"/>
@@ -2600,13 +2662,14 @@
       </c>
       <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>Foto: esquina 4 (si es accesible)</t>
-        </is>
-      </c>
-      <c r="K63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Foto: esquina 3 (si es accesible)</t>
+        </is>
+      </c>
       <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2616,39 +2679,28 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>foto_grieta</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>foto_esquina_4</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>${tipo_inspeccion} != 'no_inspeccionada'</t>
-        </is>
-      </c>
+      <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>max-pixels=2048</t>
+          <t>max-pixels=1600</t>
         </is>
       </c>
       <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>Foto: peor grieta, de cerca</t>
-        </is>
-      </c>
+      <c r="J64" t="inlineStr"/>
       <c r="K64" t="inlineStr">
         <is>
-          <t>Poner una moneda junto a la grieta como referencia de escala</t>
+          <t>Foto: esquina 4 (si es accesible)</t>
         </is>
       </c>
       <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2658,7 +2710,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>foto_columnas</t>
+          <t>foto_grieta</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2675,18 +2727,62 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>max-pixels=1600</t>
+          <t>max-pixels=2048</t>
         </is>
       </c>
       <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr">
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Foto: peor grieta, de cerca</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Poner una moneda junto a la grieta como referencia de escala</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>foto_columnas</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>${tipo_inspeccion} != 'no_inspeccionada'</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>max-pixels=1600</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr">
         <is>
           <t>Foto: columnas del primer piso</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>